<commit_message>
Fixed Bioc submission issues
</commit_message>
<xml_diff>
--- a/inst/extdata/ega_full_template_v2.xlsx
+++ b/inst/extdata/ega_full_template_v2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/igor/_DBM/projects/rega_package/Rega/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A18B514A-C117-5540-9888-E783F5F5DA7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CA69F79-0914-8E45-A8D5-38464F149170}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51200" yWindow="9920" windowWidth="30240" windowHeight="18880" xr2:uid="{C6701382-EF30-1B43-A607-1356FE361260}"/>
+    <workbookView xWindow="51200" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{C6701382-EF30-1B43-A607-1356FE361260}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="7" r:id="rId1"/>
@@ -669,7 +669,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="453">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="451">
   <si>
     <t>Description</t>
   </si>
@@ -1176,12 +1176,6 @@
   </si>
   <si>
     <t>EGA Inbox Relative Path</t>
-  </si>
-  <si>
-    <t>Absolute Path in sciCORE</t>
-  </si>
-  <si>
-    <t>EGAP50000000107</t>
   </si>
   <si>
     <t>* Run</t>
@@ -2054,9 +2048,6 @@
   </si>
   <si>
     <t>If you wish to add any of these to your submission, please create an appropriate entry in one of these 3 sheets and you will be able to select in from a dropdown menu afterwards.</t>
-  </si>
-  <si>
-    <t>For each dataset, you need to link to a med-dac policy, typically EGAP50000000107.</t>
   </si>
   <si>
     <t>Here you have to specify how the experiment was done (Instrument model, design name (e.g. "TruSeq Rna-Seq"), library type,...).</t>
@@ -2280,6 +2271,9 @@
   </si>
   <si>
     <t>Files cannot be reused among the different Runs. Each file can only be associated to one Run.</t>
+  </si>
+  <si>
+    <t>For each dataset, you need to link to a policy.</t>
   </si>
 </sst>
 </file>
@@ -3070,33 +3064,33 @@
   <sheetData>
     <row r="1" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="A1" s="38" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="18" x14ac:dyDescent="0.2"/>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="39" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="B4" s="5" t="s">
-        <v>443</v>
+        <v>440</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="B5" s="5" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="B6" s="5" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="B7" s="5" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="18" x14ac:dyDescent="0.2"/>
@@ -3115,55 +3109,55 @@
     </row>
     <row r="18" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="B18" s="5" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="B19" s="5" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="B20" s="5" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="18" x14ac:dyDescent="0.2"/>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" s="39" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" s="39"/>
       <c r="B23" s="5" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="B24" s="5" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="B25" s="5" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="B26" s="5" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="18" x14ac:dyDescent="0.2"/>
     <row r="28" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="39" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="B29" s="5" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="18" x14ac:dyDescent="0.2"/>
@@ -3174,17 +3168,17 @@
     </row>
     <row r="32" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="B32" s="9" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="18" x14ac:dyDescent="0.2">
       <c r="B33" s="5" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="18" x14ac:dyDescent="0.2">
       <c r="B34" s="9" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="18" x14ac:dyDescent="0.2"/>
@@ -3195,12 +3189,12 @@
     </row>
     <row r="37" spans="1:4" ht="18" x14ac:dyDescent="0.2">
       <c r="B37" s="5" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="18" x14ac:dyDescent="0.2">
       <c r="B38" s="5" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="18" x14ac:dyDescent="0.2"/>
@@ -3211,25 +3205,25 @@
     </row>
     <row r="41" spans="1:4" ht="18" x14ac:dyDescent="0.2">
       <c r="B41" s="9" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="18" x14ac:dyDescent="0.2">
       <c r="B42" s="9" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="18" x14ac:dyDescent="0.2">
       <c r="B43" s="5" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="18" x14ac:dyDescent="0.2">
       <c r="B44" s="44" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="D44" s="5" t="s">
         <v>2</v>
@@ -3238,7 +3232,7 @@
     <row r="45" spans="1:4" ht="18" x14ac:dyDescent="0.2">
       <c r="B45" s="44"/>
       <c r="C45" s="5" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="D45" s="5" t="s">
         <v>3</v>
@@ -3247,7 +3241,7 @@
     <row r="46" spans="1:4" ht="18" x14ac:dyDescent="0.2">
       <c r="B46" s="44"/>
       <c r="C46" s="5" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="D46" s="5" t="s">
         <v>1</v>
@@ -3264,12 +3258,12 @@
     </row>
     <row r="49" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="B49" s="5" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="B50" s="5" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="18" x14ac:dyDescent="0.2">
@@ -3277,38 +3271,38 @@
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A52" s="39" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="B52" s="40"/>
     </row>
     <row r="53" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="B53" s="5" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="B54" s="5" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="B55" s="5" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="B56" s="5" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="B57" s="5" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="B58" s="5" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
     </row>
     <row r="59" spans="1:2" ht="18" x14ac:dyDescent="0.2"/>
@@ -3319,76 +3313,76 @@
     </row>
     <row r="61" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="B61" s="9" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
     </row>
     <row r="62" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="B62" s="9" t="s">
-        <v>437</v>
+        <v>450</v>
       </c>
     </row>
     <row r="63" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="B63" s="9" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
     </row>
     <row r="64" spans="1:2" ht="18" x14ac:dyDescent="0.2"/>
     <row r="65" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A65" s="39" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
     </row>
     <row r="66" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="B66" s="5" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
     </row>
     <row r="67" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="B67" s="5" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
     </row>
     <row r="68" spans="1:2" ht="18" x14ac:dyDescent="0.2"/>
     <row r="69" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="39" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
     </row>
     <row r="70" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="B70" s="5" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
     </row>
     <row r="71" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="B71" s="5" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
     </row>
     <row r="72" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="B72" s="5" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
     </row>
     <row r="73" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="B73" s="5" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
     </row>
     <row r="74" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="A74" s="42"/>
       <c r="B74" s="42" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
     </row>
     <row r="75" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="A75" s="43"/>
       <c r="B75" s="43" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
     </row>
     <row r="76" spans="1:2" ht="18" x14ac:dyDescent="0.2">
       <c r="B76" s="5" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
     </row>
   </sheetData>
@@ -3416,7 +3410,7 @@
   <sheetData>
     <row r="1" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="21" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="B1" s="22" t="s">
         <v>10</v>
@@ -3424,10 +3418,10 @@
     </row>
     <row r="2" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="21" t="s">
+        <v>380</v>
+      </c>
+      <c r="B2" s="22" t="s">
         <v>382</v>
-      </c>
-      <c r="B2" s="22" t="s">
-        <v>384</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
@@ -3444,37 +3438,37 @@
     </row>
     <row r="5" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="21" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B5" s="22"/>
     </row>
     <row r="6" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="23" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B6" s="22"/>
     </row>
     <row r="7" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="21" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B7" s="22"/>
     </row>
     <row r="8" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="21" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B8" s="22"/>
     </row>
     <row r="9" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="21" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="B9" s="22"/>
     </row>
     <row r="10" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="23" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="B10" s="22"/>
     </row>
@@ -3494,16 +3488,16 @@
     </row>
     <row r="13" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="23" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B13" s="22"/>
     </row>
     <row r="14" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="23" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="B14" s="22" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
   </sheetData>
@@ -3603,7 +3597,7 @@
   <sheetData>
     <row r="1" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="15" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>11</v>
@@ -3623,11 +3617,9 @@
     </row>
     <row r="4" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="15" t="s">
-        <v>172</v>
-      </c>
-      <c r="B4" s="6" t="s">
         <v>170</v>
       </c>
+      <c r="B4" s="6"/>
     </row>
     <row r="5" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="20" t="s">
@@ -3651,7 +3643,7 @@
     </row>
     <row r="8" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="20" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="B8" s="6"/>
     </row>
@@ -3712,13 +3704,13 @@
   <sheetData>
     <row r="1" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="32" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B1" s="32" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="C1" s="32" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
@@ -3751,13 +3743,13 @@
   <sheetData>
     <row r="1" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="32" t="s">
+        <v>174</v>
+      </c>
+      <c r="B1" s="32" t="s">
+        <v>175</v>
+      </c>
+      <c r="C1" s="32" t="s">
         <v>176</v>
-      </c>
-      <c r="B1" s="32" t="s">
-        <v>177</v>
-      </c>
-      <c r="C1" s="32" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
@@ -3784,13 +3776,13 @@
   <sheetData>
     <row r="1" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="32" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B1" s="32" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C1" s="32" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
@@ -3825,46 +3817,46 @@
   <sheetData>
     <row r="1" spans="1:14" s="34" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="34" t="s">
+        <v>387</v>
+      </c>
+      <c r="B1" s="34" t="s">
+        <v>388</v>
+      </c>
+      <c r="C1" s="34" t="s">
         <v>389</v>
       </c>
-      <c r="B1" s="34" t="s">
+      <c r="D1" s="34" t="s">
         <v>390</v>
       </c>
-      <c r="C1" s="34" t="s">
+      <c r="E1" s="34" t="s">
         <v>391</v>
       </c>
-      <c r="D1" s="34" t="s">
+      <c r="F1" s="34" t="s">
         <v>392</v>
       </c>
-      <c r="E1" s="34" t="s">
+      <c r="G1" s="34" t="s">
         <v>393</v>
       </c>
-      <c r="F1" s="34" t="s">
+      <c r="H1" s="34" t="s">
         <v>394</v>
       </c>
-      <c r="G1" s="34" t="s">
+      <c r="I1" s="34" t="s">
         <v>395</v>
       </c>
-      <c r="H1" s="34" t="s">
+      <c r="J1" s="34" t="s">
         <v>396</v>
       </c>
-      <c r="I1" s="34" t="s">
+      <c r="K1" s="34" t="s">
         <v>397</v>
       </c>
-      <c r="J1" s="34" t="s">
+      <c r="L1" s="34" t="s">
         <v>398</v>
       </c>
-      <c r="K1" s="34" t="s">
+      <c r="M1" s="34" t="s">
         <v>399</v>
       </c>
-      <c r="L1" s="34" t="s">
+      <c r="N1" s="34" t="s">
         <v>400</v>
-      </c>
-      <c r="M1" s="34" t="s">
-        <v>401</v>
-      </c>
-      <c r="N1" s="34" t="s">
-        <v>402</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
@@ -3878,7 +3870,7 @@
         <v>135</v>
       </c>
       <c r="D2" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="E2" t="s">
         <v>29</v>
@@ -3893,7 +3885,7 @@
         <v>79</v>
       </c>
       <c r="I2" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="J2" t="s">
         <v>109</v>
@@ -3902,10 +3894,10 @@
         <v>112</v>
       </c>
       <c r="L2" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="M2" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="N2" t="s">
         <v>112</v>
@@ -3922,7 +3914,7 @@
         <v>136</v>
       </c>
       <c r="D3" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="E3" t="s">
         <v>30</v>
@@ -3937,7 +3929,7 @@
         <v>80</v>
       </c>
       <c r="I3" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="J3" t="s">
         <v>110</v>
@@ -3946,10 +3938,10 @@
         <v>113</v>
       </c>
       <c r="L3" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="M3" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="N3" t="s">
         <v>114</v>
@@ -3966,7 +3958,7 @@
         <v>137</v>
       </c>
       <c r="D4" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="F4" t="s">
         <v>33</v>
@@ -3978,7 +3970,7 @@
         <v>81</v>
       </c>
       <c r="I4" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="J4" t="s">
         <v>111</v>
@@ -3987,10 +3979,10 @@
         <v>114</v>
       </c>
       <c r="L4" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="M4" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="N4" t="s">
         <v>115</v>
@@ -4007,7 +3999,7 @@
         <v>138</v>
       </c>
       <c r="D5" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F5" t="s">
         <v>34</v>
@@ -4019,16 +4011,16 @@
         <v>82</v>
       </c>
       <c r="I5" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="K5" t="s">
         <v>115</v>
       </c>
       <c r="L5" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="M5" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="N5" t="s">
         <v>120</v>
@@ -4039,7 +4031,7 @@
         <v>18</v>
       </c>
       <c r="D6" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F6" t="s">
         <v>35</v>
@@ -4051,16 +4043,16 @@
         <v>83</v>
       </c>
       <c r="I6" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="K6" t="s">
         <v>116</v>
       </c>
       <c r="L6" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="M6" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="N6" t="s">
         <v>121</v>
@@ -4071,7 +4063,7 @@
         <v>19</v>
       </c>
       <c r="D7" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="F7" t="s">
         <v>36</v>
@@ -4083,16 +4075,16 @@
         <v>84</v>
       </c>
       <c r="I7" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="K7" t="s">
         <v>117</v>
       </c>
       <c r="L7" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="M7" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="N7" t="s">
         <v>122</v>
@@ -4103,7 +4095,7 @@
         <v>20</v>
       </c>
       <c r="D8" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="F8" t="s">
         <v>37</v>
@@ -4115,16 +4107,16 @@
         <v>85</v>
       </c>
       <c r="I8" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="K8" t="s">
         <v>118</v>
       </c>
       <c r="L8" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="M8" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="N8" t="s">
         <v>123</v>
@@ -4135,7 +4127,7 @@
         <v>21</v>
       </c>
       <c r="D9" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="F9" t="s">
         <v>38</v>
@@ -4147,16 +4139,16 @@
         <v>86</v>
       </c>
       <c r="I9" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="K9" t="s">
         <v>119</v>
       </c>
       <c r="L9" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="M9" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="N9" t="s">
         <v>124</v>
@@ -4167,7 +4159,7 @@
         <v>22</v>
       </c>
       <c r="D10" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="F10" t="s">
         <v>39</v>
@@ -4179,13 +4171,13 @@
         <v>87</v>
       </c>
       <c r="I10" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="L10" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="M10" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="N10" t="s">
         <v>125</v>
@@ -4196,7 +4188,7 @@
         <v>23</v>
       </c>
       <c r="D11" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="F11" t="s">
         <v>40</v>
@@ -4205,13 +4197,13 @@
         <v>88</v>
       </c>
       <c r="I11" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="L11" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="M11" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="N11" t="s">
         <v>126</v>
@@ -4222,7 +4214,7 @@
         <v>24</v>
       </c>
       <c r="D12" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="F12" t="s">
         <v>41</v>
@@ -4231,13 +4223,13 @@
         <v>89</v>
       </c>
       <c r="I12" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="L12" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="M12" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="N12" t="s">
         <v>127</v>
@@ -4248,7 +4240,7 @@
         <v>25</v>
       </c>
       <c r="D13" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="F13" t="s">
         <v>42</v>
@@ -4257,10 +4249,10 @@
         <v>90</v>
       </c>
       <c r="L13" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="M13" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="N13" t="s">
         <v>128</v>
@@ -4271,7 +4263,7 @@
         <v>26</v>
       </c>
       <c r="D14" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="F14" t="s">
         <v>43</v>
@@ -4280,10 +4272,10 @@
         <v>91</v>
       </c>
       <c r="L14" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="M14" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="N14" t="s">
         <v>129</v>
@@ -4294,7 +4286,7 @@
         <v>27</v>
       </c>
       <c r="D15" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="F15" t="s">
         <v>44</v>
@@ -4303,10 +4295,10 @@
         <v>92</v>
       </c>
       <c r="L15" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="M15" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="N15" t="s">
         <v>130</v>
@@ -4314,7 +4306,7 @@
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="D16" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="F16" t="s">
         <v>45</v>
@@ -4323,15 +4315,15 @@
         <v>93</v>
       </c>
       <c r="L16" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="M16" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
     </row>
     <row r="17" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D17" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="F17" t="s">
         <v>46</v>
@@ -4340,15 +4332,15 @@
         <v>94</v>
       </c>
       <c r="L17" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="M17" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="18" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D18" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="F18" t="s">
         <v>47</v>
@@ -4357,15 +4349,15 @@
         <v>95</v>
       </c>
       <c r="L18" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="M18" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="19" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D19" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="F19" t="s">
         <v>48</v>
@@ -4374,15 +4366,15 @@
         <v>49</v>
       </c>
       <c r="L19" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="M19" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="20" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D20" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="F20" t="s">
         <v>49</v>
@@ -4391,15 +4383,15 @@
         <v>96</v>
       </c>
       <c r="L20" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="M20" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="21" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D21" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="F21" t="s">
         <v>50</v>
@@ -4408,15 +4400,15 @@
         <v>97</v>
       </c>
       <c r="L21" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="M21" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="22" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D22" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="F22" t="s">
         <v>51</v>
@@ -4425,15 +4417,15 @@
         <v>98</v>
       </c>
       <c r="L22" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="M22" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="23" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D23" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="F23" t="s">
         <v>52</v>
@@ -4442,15 +4434,15 @@
         <v>99</v>
       </c>
       <c r="L23" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="M23" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
     <row r="24" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D24" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="F24" t="s">
         <v>53</v>
@@ -4459,15 +4451,15 @@
         <v>100</v>
       </c>
       <c r="L24" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="M24" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="25" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D25" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F25" t="s">
         <v>54</v>
@@ -4476,15 +4468,15 @@
         <v>101</v>
       </c>
       <c r="L25" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="M25" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="26" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D26" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="F26" t="s">
         <v>55</v>
@@ -4493,15 +4485,15 @@
         <v>102</v>
       </c>
       <c r="L26" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="M26" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="27" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D27" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="F27" t="s">
         <v>56</v>
@@ -4510,15 +4502,15 @@
         <v>103</v>
       </c>
       <c r="L27" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="M27" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="28" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D28" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="F28" t="s">
         <v>57</v>
@@ -4527,15 +4519,15 @@
         <v>104</v>
       </c>
       <c r="L28" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="M28" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="29" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D29" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F29" t="s">
         <v>58</v>
@@ -4544,15 +4536,15 @@
         <v>105</v>
       </c>
       <c r="L29" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="M29" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="30" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D30" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="F30" t="s">
         <v>59</v>
@@ -4561,15 +4553,15 @@
         <v>106</v>
       </c>
       <c r="L30" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="M30" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
     <row r="31" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D31" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="F31" t="s">
         <v>60</v>
@@ -4578,12 +4570,12 @@
         <v>107</v>
       </c>
       <c r="M31" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="32" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D32" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="F32" t="s">
         <v>61</v>
@@ -4592,411 +4584,411 @@
         <v>108</v>
       </c>
       <c r="M32" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="33" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D33" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="F33" t="s">
         <v>62</v>
       </c>
       <c r="M33" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
     </row>
     <row r="34" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D34" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="F34" t="s">
         <v>63</v>
       </c>
       <c r="M34" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
     </row>
     <row r="35" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D35" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="F35" t="s">
         <v>64</v>
       </c>
       <c r="M35" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="36" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D36" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="F36" t="s">
         <v>65</v>
       </c>
       <c r="M36" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
     </row>
     <row r="37" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D37" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="F37" t="s">
         <v>66</v>
       </c>
       <c r="M37" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
     </row>
     <row r="38" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D38" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="F38" t="s">
         <v>67</v>
       </c>
       <c r="M38" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="39" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D39" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="F39" t="s">
         <v>68</v>
       </c>
       <c r="M39" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
     </row>
     <row r="40" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D40" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="F40" t="s">
         <v>69</v>
       </c>
       <c r="M40" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
     </row>
     <row r="41" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D41" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="F41" t="s">
         <v>70</v>
       </c>
       <c r="M41" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
     </row>
     <row r="42" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D42" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="F42" t="s">
         <v>71</v>
       </c>
       <c r="M42" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
     </row>
     <row r="43" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D43" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="M43" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="44" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D44" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="M44" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
     </row>
     <row r="45" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D45" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="M45" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
     </row>
     <row r="46" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D46" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="M46" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
     </row>
     <row r="47" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D47" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="M47" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
     </row>
     <row r="48" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D48" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="M48" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
     </row>
     <row r="49" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D49" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="M49" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
     </row>
     <row r="50" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D50" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="M50" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
     </row>
     <row r="51" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D51" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="M51" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
     </row>
     <row r="52" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D52" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="M52" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
     </row>
     <row r="53" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D53" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="M53" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
     </row>
     <row r="54" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D54" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="M54" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="55" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D55" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="M55" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
     </row>
     <row r="56" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D56" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="M56" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
     </row>
     <row r="57" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D57" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="M57" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
     </row>
     <row r="58" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D58" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="M58" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="59" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D59" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="M59" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
     </row>
     <row r="60" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D60" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="M60" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
     </row>
     <row r="61" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D61" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="M61" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
     </row>
     <row r="62" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D62" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="M62" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
     </row>
     <row r="63" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D63" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="M63" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="64" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D64" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="M64" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
     </row>
     <row r="65" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D65" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="M65" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
     </row>
     <row r="66" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D66" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="M66" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
     </row>
     <row r="67" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D67" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="M67" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
     </row>
     <row r="68" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D68" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="M68" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
     </row>
     <row r="69" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D69" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="M69" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
     </row>
     <row r="70" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D70" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="M70" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
     </row>
     <row r="71" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D71" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="M71" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="72" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D72" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="M72" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="73" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D73" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="M73" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
     </row>
     <row r="74" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D74" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="M74" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="75" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D75" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="M75" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
     </row>
     <row r="76" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D76" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="77" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D77" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="78" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D78" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
     </row>
     <row r="79" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D79" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="80" spans="4:13" x14ac:dyDescent="0.2">
       <c r="D80" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
     </row>
     <row r="81" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D81" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
     </row>
   </sheetData>
@@ -5035,7 +5027,7 @@
         <v>6</v>
       </c>
       <c r="F1" s="26" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
@@ -5049,13 +5041,13 @@
         <v>11</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
     </row>
   </sheetData>
@@ -5069,106 +5061,82 @@
   <sheetPr>
     <tabColor theme="9" tint="0.39997558519241921"/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="89" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="122" style="3" customWidth="1"/>
-    <col min="3" max="3" width="41.83203125" style="3" customWidth="1"/>
-    <col min="4" max="16384" width="10.83203125" style="1"/>
+    <col min="2" max="2" width="41.83203125" style="3" customWidth="1"/>
+    <col min="3" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="2" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" s="2" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="13" t="s">
         <v>167</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>169</v>
-      </c>
-      <c r="C1" s="13" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="16"/>
-    </row>
-    <row r="3" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B2" s="16"/>
+    </row>
+    <row r="3" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3"/>
-      <c r="B3" s="1"/>
-    </row>
-    <row r="4" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="4" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4"/>
-      <c r="B4" s="1"/>
-    </row>
-    <row r="5" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="5" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5"/>
-      <c r="B5" s="1"/>
-    </row>
-    <row r="6" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="6" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6"/>
-      <c r="B6" s="1"/>
-    </row>
-    <row r="7" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="7" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7"/>
-      <c r="B7" s="1"/>
-    </row>
-    <row r="8" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="8" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8"/>
-      <c r="B8" s="1"/>
-    </row>
-    <row r="9" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="9" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9"/>
-      <c r="B9" s="1"/>
-    </row>
-    <row r="10" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="10" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10"/>
-      <c r="B10" s="1"/>
-    </row>
-    <row r="11" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="11" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11"/>
-      <c r="B11" s="1"/>
-    </row>
-    <row r="12" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="12" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12"/>
-      <c r="B12" s="1"/>
-    </row>
-    <row r="13" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="13" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13"/>
-      <c r="B13" s="1"/>
-    </row>
-    <row r="14" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="14" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14"/>
-      <c r="B14" s="1"/>
-    </row>
-    <row r="15" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="15" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15"/>
-      <c r="B15" s="1"/>
-    </row>
-    <row r="16" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="16" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16"/>
-      <c r="B16" s="1"/>
-    </row>
-    <row r="17" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="17" spans="1:1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17"/>
-      <c r="B17" s="1"/>
-    </row>
-    <row r="18" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="18" spans="1:1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18"/>
-      <c r="B18" s="1"/>
-    </row>
-    <row r="19" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="19" spans="1:1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19"/>
-      <c r="B19" s="1"/>
-    </row>
-    <row r="20" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="20" spans="1:1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20"/>
-      <c r="B20" s="1"/>
-    </row>
-    <row r="21" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="21" spans="1:1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21"/>
-      <c r="B21" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5180,125 +5148,101 @@
   <sheetPr>
     <tabColor theme="9" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="61.33203125" style="25" customWidth="1"/>
-    <col min="2" max="2" width="112.5" style="25" customWidth="1"/>
-    <col min="3" max="3" width="29.5" style="25" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="10.83203125" style="25"/>
+    <col min="2" max="2" width="29.5" style="25" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="10.83203125" style="25"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="24" t="s">
         <v>167</v>
       </c>
       <c r="B1" s="24" t="s">
-        <v>169</v>
-      </c>
-      <c r="C1" s="24" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="27"/>
-    </row>
-    <row r="3" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B2" s="27"/>
+    </row>
+    <row r="3" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="28"/>
-    </row>
-    <row r="4" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B3" s="28"/>
+    </row>
+    <row r="4" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="28"/>
-    </row>
-    <row r="5" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B4" s="28"/>
+    </row>
+    <row r="5" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="28"/>
-    </row>
-    <row r="6" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B5" s="28"/>
+    </row>
+    <row r="6" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="28"/>
-    </row>
-    <row r="7" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B6" s="28"/>
+    </row>
+    <row r="7" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="28"/>
-    </row>
-    <row r="8" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B7" s="28"/>
+    </row>
+    <row r="8" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="28"/>
-    </row>
-    <row r="9" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B8" s="28"/>
+    </row>
+    <row r="9" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="28"/>
-    </row>
-    <row r="10" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B9" s="28"/>
+    </row>
+    <row r="10" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="28"/>
-    </row>
-    <row r="11" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B10" s="28"/>
+    </row>
+    <row r="11" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="28"/>
-    </row>
-    <row r="12" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B11" s="28"/>
+    </row>
+    <row r="12" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="28"/>
-    </row>
-    <row r="13" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B12" s="28"/>
+    </row>
+    <row r="13" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="28"/>
-    </row>
-    <row r="14" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B13" s="28"/>
+    </row>
+    <row r="14" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="28"/>
-    </row>
-    <row r="15" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B14" s="28"/>
+    </row>
+    <row r="15" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="28"/>
-    </row>
-    <row r="16" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B15" s="28"/>
+    </row>
+    <row r="16" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="28"/>
-    </row>
-    <row r="17" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B16" s="28"/>
+    </row>
+    <row r="17" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="28"/>
-    </row>
-    <row r="18" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B17" s="28"/>
+    </row>
+    <row r="18" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="28"/>
-    </row>
-    <row r="19" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B18" s="28"/>
+    </row>
+    <row r="19" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="28"/>
-    </row>
-    <row r="20" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B19" s="28"/>
+    </row>
+    <row r="20" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="28"/>
-    </row>
-    <row r="21" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B20" s="28"/>
+    </row>
+    <row r="21" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="28"/>
+      <c r="B21" s="28"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5333,7 +5277,7 @@
     </row>
     <row r="3" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="23" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B3" s="22"/>
     </row>
@@ -5371,7 +5315,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="17" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="B1" s="7" t="s">
         <v>10</v>
@@ -5510,7 +5454,7 @@
     </row>
     <row r="2" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="10" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -5575,7 +5519,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="15" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="B1" s="6" t="s">
         <v>10</v>
@@ -5584,7 +5528,7 @@
     </row>
     <row r="2" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="15" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="B2" s="8" t="s">
         <v>12</v>
@@ -5743,10 +5687,10 @@
   <sheetData>
     <row r="1" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="30" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B1" s="29" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="C1" s="14" t="s">
         <v>166</v>
@@ -5758,7 +5702,7 @@
         <v>144</v>
       </c>
       <c r="F1" s="14" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="G1" s="14" t="s">
         <v>8</v>
@@ -5772,10 +5716,10 @@
         <v>12</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="E2" s="41"/>
       <c r="F2" s="41"/>

</xml_diff>

<commit_message>
New submission template and API yaml creation.
</commit_message>
<xml_diff>
--- a/inst/extdata/ega_full_template_v2.xlsx
+++ b/inst/extdata/ega_full_template_v2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/igor/_DBM/projects/rega_package/Rega/inst/extdata/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/igor/_DBM/programming/packages/rega_package/Rega/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CA69F79-0914-8E45-A8D5-38464F149170}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41CE7284-3BBE-0C4D-A5A4-FECE84DDE21F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51200" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{C6701382-EF30-1B43-A607-1356FE361260}"/>
+    <workbookView xWindow="12740" yWindow="7120" windowWidth="36940" windowHeight="19880" xr2:uid="{C6701382-EF30-1B43-A607-1356FE361260}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="7" r:id="rId1"/>

</xml_diff>